<commit_message>
Fix Riepilogo Generale: tolte colonne vuote, riferimenti diretti come template (D/E), colonna K budget
</commit_message>
<xml_diff>
--- a/Monitoraggio_ORE18_TECNINF_SPA_30-09-2026.xlsx
+++ b/Monitoraggio_ORE18_TECNINF_SPA_30-09-2026.xlsx
@@ -317,39 +317,39 @@
     <author>Monitoring</author>
   </authors>
   <commentList>
-    <comment ref="J2" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
         <t>Somma delle ore effettive mensili (formule dai fogli mese).</t>
       </text>
     </comment>
-    <comment ref="K2" authorId="0" shapeId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
         <t>Somma degli eccessi mensili (weekend + dopo soglia serale + mattutino + oltre cap 8h/giorno).</t>
       </text>
     </comment>
-    <comment ref="L2" authorId="0" shapeId="0">
+    <comment ref="F2" authorId="0" shapeId="0">
       <text>
         <t>% COPERTURA NON compensativa = MIN((Ore Maturate in ore) / 75, somma_cappata / somma_attese), cappata al 100%. somma_cappata = SUM delle % Dettaglio del percorso del discente * rispettive attese: il 100% scatta solo se TUTTI i corsi attesi sono al 100%. Formula: =IF(75=0,0,MIN((D*24)/150,1)).</t>
       </text>
     </comment>
-    <comment ref="M2" authorId="0" shapeId="0">
+    <comment ref="G2" authorId="0" shapeId="0">
       <text>
         <t>Titoli dei corsi del percorso del discente INIZIATI (ore &gt; 0) e NON al 100% (stessi titoli canonici delle intestazioni dei fogli 'Dettaglio - &lt;base&gt;', testo statico senza formule).</t>
       </text>
     </comment>
-    <comment ref="N2" authorId="0" shapeId="0">
+    <comment ref="H2" authorId="0" shapeId="0">
       <text>
         <t>Costo orario retributivo del discente, dal file costi aziendale.
 'N/D' se il Codice Fiscale non e' presente nel file costi.</t>
       </text>
     </comment>
-    <comment ref="O2" authorId="0" shapeId="0">
+    <comment ref="I2" authorId="0" shapeId="0">
       <text>
         <t>Costo orario contributivo del discente, dal file costi aziendale.
 'N/D' se il Codice Fiscale non e' presente nel file costi.</t>
       </text>
     </comment>
-    <comment ref="P2" authorId="0" shapeId="0">
+    <comment ref="J2" authorId="0" shapeId="0">
       <text>
         <t>Finanziamento = (Quota 80% + Costo orario Contributivo) * MIN(Ore Maturate, 75).</t>
       </text>
@@ -2727,20 +2727,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="130.28515625" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col hidden="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="130.28515625" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.1" customHeight="1">
@@ -2766,44 +2766,44 @@
           <t>Percorso Formativo</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Totale
 Ore Maturate</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Ore Tolte
 (totali)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>%
 copertura</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Corsi da
 finire</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Quota Retr.
 al 80%
 (€/h)</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Costo orario
 contributivo</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Finanziamento</t>
         </is>
@@ -2825,31 +2825,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J3" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PZLWLM96A16Z504F",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PZLWLM96A16Z504F",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PZLWLM96A16Z504F",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PZLWLM96A16Z504F",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PZLWLM96A16Z504F",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PZLWLM96A16Z504F",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K3" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PZLWLM96A16Z504F",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PZLWLM96A16Z504F",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PZLWLM96A16Z504F",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PZLWLM96A16Z504F",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PZLWLM96A16Z504F",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PZLWLM96A16Z504F",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L3" s="6">
-        <f>IF(75=0,0,MIN((J3*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="D3" s="5">
+        <f>'Aprile 2026'!AH4+'Maggio 2026'!AI4+'Giugno 2026'!AH4+'Luglio 2026'!AI4+'Agosto 2026'!AI4+'Settembre 2026'!AH4</f>
+        <v/>
+      </c>
+      <c r="E3" s="5">
+        <f>'Aprile 2026'!AJ4+'Maggio 2026'!AK4+'Giugno 2026'!AJ4+'Luglio 2026'!AK4+'Agosto 2026'!AK4+'Settembre 2026'!AJ4</f>
+        <v/>
+      </c>
+      <c r="F3" s="6">
+        <f>IF(75=0,0,MIN((D3*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; I sistemi operativi; Linguaggi di programmazione</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P3" s="7">
-        <f>(N3+O3)*J3*24</f>
+      <c r="J3" s="7">
+        <f>(H3+I3)*D3*24</f>
         <v/>
       </c>
     </row>
@@ -2869,31 +2869,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J4" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("BDALSN01R03H501Z",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("BDALSN01R03H501Z",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("BDALSN01R03H501Z",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("BDALSN01R03H501Z",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("BDALSN01R03H501Z",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("BDALSN01R03H501Z",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K4" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("BDALSN01R03H501Z",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("BDALSN01R03H501Z",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("BDALSN01R03H501Z",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("BDALSN01R03H501Z",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("BDALSN01R03H501Z",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("BDALSN01R03H501Z",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="6">
-        <f>IF(75=0,0,MIN((J4*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="D4" s="5">
+        <f>'Aprile 2026'!AH5+'Maggio 2026'!AI5+'Giugno 2026'!AH5+'Luglio 2026'!AI5+'Agosto 2026'!AI5+'Settembre 2026'!AH5</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>'Aprile 2026'!AJ5+'Maggio 2026'!AK5+'Giugno 2026'!AJ5+'Luglio 2026'!AK5+'Agosto 2026'!AK5+'Settembre 2026'!AJ5</f>
+        <v/>
+      </c>
+      <c r="F4" s="6">
+        <f>IF(75=0,0,MIN((D4*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>I Big data in ambito finanziario; Deep Learning e reti neurali; Sicurezza e Password Management</t>
         </is>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P4" s="7">
-        <f>(N4+O4)*J4*24</f>
+      <c r="J4" s="7">
+        <f>(H4+I4)*D4*24</f>
         <v/>
       </c>
     </row>
@@ -2913,31 +2913,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J5" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("BDNHHM97H19H501Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("BDNHHM97H19H501Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("BDNHHM97H19H501Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("BDNHHM97H19H501Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("BDNHHM97H19H501Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("BDNHHM97H19H501Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K5" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("BDNHHM97H19H501Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("BDNHHM97H19H501Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("BDNHHM97H19H501Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("BDNHHM97H19H501Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("BDNHHM97H19H501Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("BDNHHM97H19H501Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L5" s="6">
-        <f>IF(75=0,0,MIN((J5*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="D5" s="5">
+        <f>'Aprile 2026'!AH6+'Maggio 2026'!AI6+'Giugno 2026'!AH6+'Luglio 2026'!AI6+'Agosto 2026'!AI6+'Settembre 2026'!AH6</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>'Aprile 2026'!AJ6+'Maggio 2026'!AK6+'Giugno 2026'!AJ6+'Luglio 2026'!AK6+'Agosto 2026'!AK6+'Settembre 2026'!AJ6</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>IF(75=0,0,MIN((D5*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Front end base: HTML, CSS, Bootstrap; Front end avanzato: JavaScript e jQuery</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>3.235298414499312</v>
       </c>
-      <c r="P5" s="7">
-        <f>(N5+O5)*J5*24</f>
+      <c r="J5" s="7">
+        <f>(H5+I5)*D5*24</f>
         <v/>
       </c>
     </row>
@@ -2957,31 +2957,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J6" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("BCNNDR82P16D773D",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("BCNNDR82P16D773D",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("BCNNDR82P16D773D",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("BCNNDR82P16D773D",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("BCNNDR82P16D773D",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("BCNNDR82P16D773D",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K6" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("BCNNDR82P16D773D",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("BCNNDR82P16D773D",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("BCNNDR82P16D773D",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("BCNNDR82P16D773D",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("BCNNDR82P16D773D",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("BCNNDR82P16D773D",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L6" s="6">
-        <f>IF(75=0,0,MIN((J6*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="D6" s="5">
+        <f>'Aprile 2026'!AH7+'Maggio 2026'!AI7+'Giugno 2026'!AH7+'Luglio 2026'!AI7+'Agosto 2026'!AI7+'Settembre 2026'!AH7</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>'Aprile 2026'!AJ7+'Maggio 2026'!AK7+'Giugno 2026'!AJ7+'Luglio 2026'!AK7+'Agosto 2026'!AK7+'Settembre 2026'!AJ7</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>IF(75=0,0,MIN((D6*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>I sistemi operativi; Linguaggi di programmazione; Back end base: Fondamenti di PHP; Back end avanzato: PHP MVC con Laravel</t>
         </is>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>9.304</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>5.11</v>
       </c>
-      <c r="P6" s="7">
-        <f>(N6+O6)*J6*24</f>
+      <c r="J6" s="7">
+        <f>(H6+I6)*D6*24</f>
         <v/>
       </c>
     </row>
@@ -3001,31 +3001,31 @@
           <t>Project Management per il digitale - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J7" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("BNTJTP78S54Z241U",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("BNTJTP78S54Z241U",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("BNTJTP78S54Z241U",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("BNTJTP78S54Z241U",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("BNTJTP78S54Z241U",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("BNTJTP78S54Z241U",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K7" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("BNTJTP78S54Z241U",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("BNTJTP78S54Z241U",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("BNTJTP78S54Z241U",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("BNTJTP78S54Z241U",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("BNTJTP78S54Z241U",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("BNTJTP78S54Z241U",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="6">
-        <f>IF(75=0,0,MIN((J7*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="D7" s="5">
+        <f>'Aprile 2026'!AH8+'Maggio 2026'!AI8+'Giugno 2026'!AH8+'Luglio 2026'!AI8+'Agosto 2026'!AI8+'Settembre 2026'!AH8</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>'Aprile 2026'!AJ8+'Maggio 2026'!AK8+'Giugno 2026'!AJ8+'Luglio 2026'!AK8+'Agosto 2026'!AK8+'Settembre 2026'!AJ8</f>
+        <v/>
+      </c>
+      <c r="F7" s="6">
+        <f>IF(75=0,0,MIN((D7*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>La gestione delle risorse umane; La swot analysis del personale; Fondamenti di Project Management; Leadership e Motivazione; Skills e competenze per comunicare in azienda</t>
         </is>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>13.17800930232558</v>
       </c>
-      <c r="O7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>6.56758080265642</v>
       </c>
-      <c r="P7" s="7">
-        <f>(N7+O7)*J7*24</f>
+      <c r="J7" s="7">
+        <f>(H7+I7)*D7*24</f>
         <v/>
       </c>
     </row>
@@ -3045,31 +3045,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J8" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("BTTGRG97S59G274Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("BTTGRG97S59G274Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("BTTGRG97S59G274Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("BTTGRG97S59G274Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("BTTGRG97S59G274Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("BTTGRG97S59G274Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K8" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("BTTGRG97S59G274Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("BTTGRG97S59G274Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("BTTGRG97S59G274Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("BTTGRG97S59G274Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("BTTGRG97S59G274Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("BTTGRG97S59G274Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="6">
-        <f>IF(75=0,0,MIN((J8*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="D8" s="5">
+        <f>'Aprile 2026'!AH9+'Maggio 2026'!AI9+'Giugno 2026'!AH9+'Luglio 2026'!AI9+'Agosto 2026'!AI9+'Settembre 2026'!AH9</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>'Aprile 2026'!AJ9+'Maggio 2026'!AK9+'Giugno 2026'!AJ9+'Luglio 2026'!AK9+'Agosto 2026'!AK9+'Settembre 2026'!AJ9</f>
+        <v/>
+      </c>
+      <c r="F8" s="6">
+        <f>IF(75=0,0,MIN((D8*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Introduzione ai Big Data nelle aziende; Big data e analisi predittiva; I Big data in ambito finanziario; Database relazionali e linguaggio SQL con PHP; Natural Language Processing con Python; Progettare autorizzazioni e autentificazioni; Gestione avanzata di un Database</t>
         </is>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>9.984876279069768</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>4.976207445962649</v>
       </c>
-      <c r="P8" s="7">
-        <f>(N8+O8)*J8*24</f>
+      <c r="J8" s="7">
+        <f>(H8+I8)*D8*24</f>
         <v/>
       </c>
     </row>
@@ -3089,31 +3089,31 @@
           <t>Sicurezza Informatica - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J9" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("CRBVTR94A11Z140B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("CRBVTR94A11Z140B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("CRBVTR94A11Z140B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("CRBVTR94A11Z140B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("CRBVTR94A11Z140B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("CRBVTR94A11Z140B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K9" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("CRBVTR94A11Z140B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("CRBVTR94A11Z140B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("CRBVTR94A11Z140B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("CRBVTR94A11Z140B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("CRBVTR94A11Z140B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("CRBVTR94A11Z140B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="6">
-        <f>IF(75=0,0,MIN((J9*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="D9" s="5">
+        <f>'Aprile 2026'!AH10+'Maggio 2026'!AI10+'Giugno 2026'!AH10+'Luglio 2026'!AI10+'Agosto 2026'!AI10+'Settembre 2026'!AH10</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>'Aprile 2026'!AJ10+'Maggio 2026'!AK10+'Giugno 2026'!AJ10+'Luglio 2026'!AK10+'Agosto 2026'!AK10+'Settembre 2026'!AJ10</f>
+        <v/>
+      </c>
+      <c r="F9" s="6">
+        <f>IF(75=0,0,MIN((D9*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; La Cyber Security; La Network Security; Cloud e Fog Computing; I sistemi cyber fisici; Internet delle Cose e delle Macchine; Gli attacchi tramite Ransomware</t>
         </is>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>9.858164651162792</v>
       </c>
-      <c r="O9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>4.913013289280792</v>
       </c>
-      <c r="P9" s="7">
-        <f>(N9+O9)*J9*24</f>
+      <c r="J9" s="7">
+        <f>(H9+I9)*D9*24</f>
         <v/>
       </c>
     </row>
@@ -3133,31 +3133,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J10" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("CCCNHN91D19H501W",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("CCCNHN91D19H501W",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("CCCNHN91D19H501W",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("CCCNHN91D19H501W",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("CCCNHN91D19H501W",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("CCCNHN91D19H501W",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K10" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("CCCNHN91D19H501W",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("CCCNHN91D19H501W",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("CCCNHN91D19H501W",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("CCCNHN91D19H501W",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("CCCNHN91D19H501W",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("CCCNHN91D19H501W",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="6">
-        <f>IF(75=0,0,MIN((J10*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="D10" s="5">
+        <f>'Aprile 2026'!AH11+'Maggio 2026'!AI11+'Giugno 2026'!AH11+'Luglio 2026'!AI11+'Agosto 2026'!AI11+'Settembre 2026'!AH11</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>'Aprile 2026'!AJ11+'Maggio 2026'!AK11+'Giugno 2026'!AJ11+'Luglio 2026'!AK11+'Agosto 2026'!AK11+'Settembre 2026'!AJ11</f>
+        <v/>
+      </c>
+      <c r="F10" s="6">
+        <f>IF(75=0,0,MIN((D10*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; I sistemi operativi; Applicazioni dinamiche con PHP e MySql; Back end avanzato: PHP MVC con Laravel</t>
         </is>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P10" s="7">
-        <f>(N10+O10)*J10*24</f>
+      <c r="J10" s="7">
+        <f>(H10+I10)*D10*24</f>
         <v/>
       </c>
     </row>
@@ -3177,31 +3177,31 @@
           <t>L'ufficio digitale - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J11" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("GBBMCH73R57H501G",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("GBBMCH73R57H501G",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("GBBMCH73R57H501G",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("GBBMCH73R57H501G",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("GBBMCH73R57H501G",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("GBBMCH73R57H501G",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K11" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("GBBMCH73R57H501G",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("GBBMCH73R57H501G",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("GBBMCH73R57H501G",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("GBBMCH73R57H501G",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("GBBMCH73R57H501G",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("GBBMCH73R57H501G",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="6">
-        <f>IF(75=0,0,MIN((J11*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="D11" s="5">
+        <f>'Aprile 2026'!AH12+'Maggio 2026'!AI12+'Giugno 2026'!AH12+'Luglio 2026'!AI12+'Agosto 2026'!AI12+'Settembre 2026'!AH12</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>'Aprile 2026'!AJ12+'Maggio 2026'!AK12+'Giugno 2026'!AJ12+'Luglio 2026'!AK12+'Agosto 2026'!AK12+'Settembre 2026'!AJ12</f>
+        <v/>
+      </c>
+      <c r="F11" s="6">
+        <f>IF(75=0,0,MIN((D11*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Introduzione al mondo di Microsoft office 365; Microsoft 365: Outlook desktop corso completo; Microsoft 365: Data Modeling con Power Query; Microsoft 365: elementi avanzati, suggerimenti e trucchi in PowerPoint; I sistemi informatici</t>
         </is>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>12.31637023255814</v>
       </c>
-      <c r="O11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>6.138145553425757</v>
       </c>
-      <c r="P11" s="7">
-        <f>(N11+O11)*J11*24</f>
+      <c r="J11" s="7">
+        <f>(H11+I11)*D11*24</f>
         <v/>
       </c>
     </row>
@@ -3221,31 +3221,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J12" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("LMTNIO94M03Z129S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("LMTNIO94M03Z129S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("LMTNIO94M03Z129S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("LMTNIO94M03Z129S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("LMTNIO94M03Z129S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("LMTNIO94M03Z129S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K12" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("LMTNIO94M03Z129S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("LMTNIO94M03Z129S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("LMTNIO94M03Z129S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("LMTNIO94M03Z129S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("LMTNIO94M03Z129S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("LMTNIO94M03Z129S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="6">
-        <f>IF(75=0,0,MIN((J12*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="D12" s="5">
+        <f>'Aprile 2026'!AH13+'Maggio 2026'!AI13+'Giugno 2026'!AH13+'Luglio 2026'!AI13+'Agosto 2026'!AI13+'Settembre 2026'!AH13</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>'Aprile 2026'!AJ13+'Maggio 2026'!AK13+'Giugno 2026'!AJ13+'Luglio 2026'!AK13+'Agosto 2026'!AK13+'Settembre 2026'!AJ13</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>IF(75=0,0,MIN((D12*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Big data e analisi predittiva; I Big data in ambito finanziario; Natural Language Processing con Python; Big Data Analytics con Python e Spark</t>
         </is>
       </c>
-      <c r="N12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>10.87692613953488</v>
       </c>
-      <c r="O12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>5.420755321932365</v>
       </c>
-      <c r="P12" s="7">
-        <f>(N12+O12)*J12*24</f>
+      <c r="J12" s="7">
+        <f>(H12+I12)*D12*24</f>
         <v/>
       </c>
     </row>
@@ -3265,31 +3265,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J13" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("LCUVNC85L52D976T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("LCUVNC85L52D976T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("LCUVNC85L52D976T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("LCUVNC85L52D976T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("LCUVNC85L52D976T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("LCUVNC85L52D976T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K13" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("LCUVNC85L52D976T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("LCUVNC85L52D976T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("LCUVNC85L52D976T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("LCUVNC85L52D976T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("LCUVNC85L52D976T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("LCUVNC85L52D976T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="6">
-        <f>IF(75=0,0,MIN((J13*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="D13" s="5">
+        <f>'Aprile 2026'!AH14+'Maggio 2026'!AI14+'Giugno 2026'!AH14+'Luglio 2026'!AI14+'Agosto 2026'!AI14+'Settembre 2026'!AH14</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>'Aprile 2026'!AJ14+'Maggio 2026'!AK14+'Giugno 2026'!AJ14+'Luglio 2026'!AK14+'Agosto 2026'!AK14+'Settembre 2026'!AJ14</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>IF(75=0,0,MIN((D13*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Big data e analisi predittiva</t>
         </is>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>10.42583274418605</v>
       </c>
-      <c r="O13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>3.783118027213908</v>
       </c>
-      <c r="P13" s="7">
-        <f>(N13+O13)*J13*24</f>
+      <c r="J13" s="7">
+        <f>(H13+I13)*D13*24</f>
         <v/>
       </c>
     </row>
@@ -3309,31 +3309,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J14" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("MGNLNZ97M04H501T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("MGNLNZ97M04H501T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("MGNLNZ97M04H501T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("MGNLNZ97M04H501T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("MGNLNZ97M04H501T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("MGNLNZ97M04H501T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K14" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("MGNLNZ97M04H501T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("MGNLNZ97M04H501T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("MGNLNZ97M04H501T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("MGNLNZ97M04H501T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("MGNLNZ97M04H501T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("MGNLNZ97M04H501T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="6">
-        <f>IF(75=0,0,MIN((J14*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="D14" s="5">
+        <f>'Aprile 2026'!AH15+'Maggio 2026'!AI15+'Giugno 2026'!AH15+'Luglio 2026'!AI15+'Agosto 2026'!AI15+'Settembre 2026'!AH15</f>
+        <v/>
+      </c>
+      <c r="E14" s="5">
+        <f>'Aprile 2026'!AJ15+'Maggio 2026'!AK15+'Giugno 2026'!AJ15+'Luglio 2026'!AK15+'Agosto 2026'!AK15+'Settembre 2026'!AJ15</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>IF(75=0,0,MIN((D14*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>I sistemi operativi; Front end base: HTML, CSS, Bootstrap; Front end avanzato: JavaScript e jQuery; Back end base: Fondamenti di PHP; Database relazionali e linguaggio SQL con PHP; Applicazioni dinamiche con PHP e MySql</t>
         </is>
       </c>
-      <c r="N14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>4.783158879615591</v>
       </c>
-      <c r="P14" s="7">
-        <f>(N14+O14)*J14*24</f>
+      <c r="J14" s="7">
+        <f>(H14+I14)*D14*24</f>
         <v/>
       </c>
     </row>
@@ -3353,31 +3353,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J15" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("MRNLSS75L68H501L",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("MRNLSS75L68H501L",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("MRNLSS75L68H501L",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("MRNLSS75L68H501L",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("MRNLSS75L68H501L",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("MRNLSS75L68H501L",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K15" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("MRNLSS75L68H501L",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("MRNLSS75L68H501L",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("MRNLSS75L68H501L",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("MRNLSS75L68H501L",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("MRNLSS75L68H501L",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("MRNLSS75L68H501L",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="6">
-        <f>IF(75=0,0,MIN((J15*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="D15" s="5">
+        <f>'Aprile 2026'!AH16+'Maggio 2026'!AI16+'Giugno 2026'!AH16+'Luglio 2026'!AI16+'Agosto 2026'!AI16+'Settembre 2026'!AH16</f>
+        <v/>
+      </c>
+      <c r="E15" s="5">
+        <f>'Aprile 2026'!AJ16+'Maggio 2026'!AK16+'Giugno 2026'!AJ16+'Luglio 2026'!AK16+'Agosto 2026'!AK16+'Settembre 2026'!AJ16</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>IF(75=0,0,MIN((D15*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Big data e analisi predittiva; Business Intelligence e analisi predittiva; Database relazionali e linguaggio SQL con PHP; Il Machine Learning con Python; Big Data Analytics con Python e Spark</t>
         </is>
       </c>
-      <c r="N15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>10.87692613953488</v>
       </c>
-      <c r="O15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>5.346173926583528</v>
       </c>
-      <c r="P15" s="7">
-        <f>(N15+O15)*J15*24</f>
+      <c r="J15" s="7">
+        <f>(H15+I15)*D15*24</f>
         <v/>
       </c>
     </row>
@@ -3397,31 +3397,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J16" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("MSCGLI83C04G511L",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("MSCGLI83C04G511L",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("MSCGLI83C04G511L",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("MSCGLI83C04G511L",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("MSCGLI83C04G511L",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("MSCGLI83C04G511L",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K16" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("MSCGLI83C04G511L",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("MSCGLI83C04G511L",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("MSCGLI83C04G511L",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("MSCGLI83C04G511L",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("MSCGLI83C04G511L",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("MSCGLI83C04G511L",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L16" s="6">
-        <f>IF(75=0,0,MIN((J16*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="D16" s="5">
+        <f>'Aprile 2026'!AH17+'Maggio 2026'!AI17+'Giugno 2026'!AH17+'Luglio 2026'!AI17+'Agosto 2026'!AI17+'Settembre 2026'!AH17</f>
+        <v/>
+      </c>
+      <c r="E16" s="5">
+        <f>'Aprile 2026'!AJ17+'Maggio 2026'!AK17+'Giugno 2026'!AJ17+'Luglio 2026'!AK17+'Agosto 2026'!AK17+'Settembre 2026'!AJ17</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>IF(75=0,0,MIN((D16*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Big data e analisi predittiva</t>
         </is>
       </c>
-      <c r="N16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>19.584</v>
       </c>
-      <c r="O16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>8.85</v>
       </c>
-      <c r="P16" s="7">
-        <f>(N16+O16)*J16*24</f>
+      <c r="J16" s="7">
+        <f>(H16+I16)*D16*24</f>
         <v/>
       </c>
     </row>
@@ -3441,31 +3441,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J17" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PCPMHL00R03H501G",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PCPMHL00R03H501G",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PCPMHL00R03H501G",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PCPMHL00R03H501G",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PCPMHL00R03H501G",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PCPMHL00R03H501G",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K17" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PCPMHL00R03H501G",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PCPMHL00R03H501G",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PCPMHL00R03H501G",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PCPMHL00R03H501G",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PCPMHL00R03H501G",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PCPMHL00R03H501G",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L17" s="6">
-        <f>IF(75=0,0,MIN((J17*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="D17" s="5">
+        <f>'Aprile 2026'!AH18+'Maggio 2026'!AI18+'Giugno 2026'!AH18+'Luglio 2026'!AI18+'Agosto 2026'!AI18+'Settembre 2026'!AH18</f>
+        <v/>
+      </c>
+      <c r="E17" s="5">
+        <f>'Aprile 2026'!AJ18+'Maggio 2026'!AK18+'Giugno 2026'!AJ18+'Luglio 2026'!AK18+'Agosto 2026'!AK18+'Settembre 2026'!AJ18</f>
+        <v/>
+      </c>
+      <c r="F17" s="6">
+        <f>IF(75=0,0,MIN((D17*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Linguaggi di programmazione; Back end base: Fondamenti di PHP; Applicazioni dinamiche con PHP e MySql</t>
         </is>
       </c>
-      <c r="N17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>8.746046511627904</v>
       </c>
-      <c r="O17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>2.093632948739695</v>
       </c>
-      <c r="P17" s="7">
-        <f>(N17+O17)*J17*24</f>
+      <c r="J17" s="7">
+        <f>(H17+I17)*D17*24</f>
         <v/>
       </c>
     </row>
@@ -3485,31 +3485,31 @@
           <t>Sicurezza Informatica - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J18" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PSSRRT76L56H501O",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PSSRRT76L56H501O",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PSSRRT76L56H501O",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PSSRRT76L56H501O",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PSSRRT76L56H501O",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PSSRRT76L56H501O",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K18" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PSSRRT76L56H501O",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PSSRRT76L56H501O",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PSSRRT76L56H501O",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PSSRRT76L56H501O",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PSSRRT76L56H501O",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PSSRRT76L56H501O",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L18" s="6">
-        <f>IF(75=0,0,MIN((J18*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="D18" s="5">
+        <f>'Aprile 2026'!AH19+'Maggio 2026'!AI19+'Giugno 2026'!AH19+'Luglio 2026'!AI19+'Agosto 2026'!AI19+'Settembre 2026'!AH19</f>
+        <v/>
+      </c>
+      <c r="E18" s="5">
+        <f>'Aprile 2026'!AJ19+'Maggio 2026'!AK19+'Giugno 2026'!AJ19+'Luglio 2026'!AK19+'Agosto 2026'!AK19+'Settembre 2026'!AJ19</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>IF(75=0,0,MIN((D18*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Elementi base di sicurezza informatica; Virus e Antivirus per tutti; La Cyber Security; La Network Security; Cloud e Fog Computing; I sistemi cyber fisici; Internet delle Cose e delle Macchine; Gli attacchi tramite Ransomware</t>
         </is>
       </c>
-      <c r="N18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>12.31637023255814</v>
       </c>
-      <c r="O18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>6.138145553425757</v>
       </c>
-      <c r="P18" s="7">
-        <f>(N18+O18)*J18*24</f>
+      <c r="J18" s="7">
+        <f>(H18+I18)*D18*24</f>
         <v/>
       </c>
     </row>
@@ -3529,31 +3529,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J19" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PRLGLG98M18H501X",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PRLGLG98M18H501X",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PRLGLG98M18H501X",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PRLGLG98M18H501X",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PRLGLG98M18H501X",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PRLGLG98M18H501X",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K19" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PRLGLG98M18H501X",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PRLGLG98M18H501X",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PRLGLG98M18H501X",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PRLGLG98M18H501X",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PRLGLG98M18H501X",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PRLGLG98M18H501X",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L19" s="6">
-        <f>IF(75=0,0,MIN((J19*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="D19" s="5">
+        <f>'Aprile 2026'!AH20+'Maggio 2026'!AI20+'Giugno 2026'!AH20+'Luglio 2026'!AI20+'Agosto 2026'!AI20+'Settembre 2026'!AH20</f>
+        <v/>
+      </c>
+      <c r="E19" s="5">
+        <f>'Aprile 2026'!AJ20+'Maggio 2026'!AK20+'Giugno 2026'!AJ20+'Luglio 2026'!AK20+'Agosto 2026'!AK20+'Settembre 2026'!AJ20</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>IF(75=0,0,MIN((D19*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Sicurezza e Password Management</t>
         </is>
       </c>
-      <c r="N19" s="4" t="n">
+      <c r="H19" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O19" s="4" t="n">
+      <c r="I19" s="4" t="n">
         <v>4.849907445614766</v>
       </c>
-      <c r="P19" s="7">
-        <f>(N19+O19)*J19*24</f>
+      <c r="J19" s="7">
+        <f>(H19+I19)*D19*24</f>
         <v/>
       </c>
     </row>
@@ -3573,31 +3573,31 @@
           <t>Project Management per il digitale - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J20" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("CPNRRT66D27H501V",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("CPNRRT66D27H501V",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("CPNRRT66D27H501V",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("CPNRRT66D27H501V",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("CPNRRT66D27H501V",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("CPNRRT66D27H501V",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K20" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("CPNRRT66D27H501V",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("CPNRRT66D27H501V",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("CPNRRT66D27H501V",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("CPNRRT66D27H501V",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("CPNRRT66D27H501V",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("CPNRRT66D27H501V",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L20" s="6">
-        <f>IF(75=0,0,MIN((J20*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="D20" s="5">
+        <f>'Aprile 2026'!AH21+'Maggio 2026'!AI21+'Giugno 2026'!AH21+'Luglio 2026'!AI21+'Agosto 2026'!AI21+'Settembre 2026'!AH21</f>
+        <v/>
+      </c>
+      <c r="E20" s="5">
+        <f>'Aprile 2026'!AJ21+'Maggio 2026'!AK21+'Giugno 2026'!AJ21+'Luglio 2026'!AK21+'Agosto 2026'!AK21+'Settembre 2026'!AJ21</f>
+        <v/>
+      </c>
+      <c r="F20" s="6">
+        <f>IF(75=0,0,MIN((D20*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Ottimizzare ed organizzare i meeting online; Gli approcci nel Problem Solving; Comprensione di una struttura organizzativa; Guidare un team con l'intelligenza emotiva; Fondamenti di Project Management; Predictive-Waterfall e lo sviluppo di un progetto; Comunicazione aziendale e risoluzione dei conflitti; Skills e competenze per comunicare in azienda</t>
         </is>
       </c>
-      <c r="N20" s="4" t="n">
+      <c r="H20" s="4" t="n">
         <v>14.36403013953489</v>
       </c>
-      <c r="O20" s="4" t="n">
+      <c r="I20" s="4" t="n">
         <v>7.15867607196776</v>
       </c>
-      <c r="P20" s="7">
-        <f>(N20+O20)*J20*24</f>
+      <c r="J20" s="7">
+        <f>(H20+I20)*D20*24</f>
         <v/>
       </c>
     </row>
@@ -3617,31 +3617,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J21" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PGGRRT91H07F839Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PGGRRT91H07F839Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PGGRRT91H07F839Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PGGRRT91H07F839Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PGGRRT91H07F839Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PGGRRT91H07F839Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K21" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PGGRRT91H07F839Q",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PGGRRT91H07F839Q",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PGGRRT91H07F839Q",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PGGRRT91H07F839Q",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PGGRRT91H07F839Q",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PGGRRT91H07F839Q",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L21" s="6">
-        <f>IF(75=0,0,MIN((J21*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="D21" s="5">
+        <f>'Aprile 2026'!AH22+'Maggio 2026'!AI22+'Giugno 2026'!AH22+'Luglio 2026'!AI22+'Agosto 2026'!AI22+'Settembre 2026'!AH22</f>
+        <v/>
+      </c>
+      <c r="E21" s="5">
+        <f>'Aprile 2026'!AJ22+'Maggio 2026'!AK22+'Giugno 2026'!AJ22+'Luglio 2026'!AK22+'Agosto 2026'!AK22+'Settembre 2026'!AJ22</f>
+        <v/>
+      </c>
+      <c r="F21" s="6">
+        <f>IF(75=0,0,MIN((D21*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Big Data Analytics con Python e Spark; Progettare autorizzazioni e autentificazioni; Sicurezza e Password Management</t>
         </is>
       </c>
-      <c r="N21" s="4" t="n">
+      <c r="H21" s="4" t="n">
         <v>10.87692613953488</v>
       </c>
-      <c r="O21" s="4" t="n">
+      <c r="I21" s="4" t="n">
         <v>5.420755321932365</v>
       </c>
-      <c r="P21" s="7">
-        <f>(N21+O21)*J21*24</f>
+      <c r="J21" s="7">
+        <f>(H21+I21)*D21*24</f>
         <v/>
       </c>
     </row>
@@ -3661,31 +3661,31 @@
           <t>Sicurezza Informatica - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J22" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PRSRSH87S19H501S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PRSRSH87S19H501S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PRSRSH87S19H501S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PRSRSH87S19H501S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PRSRSH87S19H501S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PRSRSH87S19H501S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K22" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PRSRSH87S19H501S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PRSRSH87S19H501S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PRSRSH87S19H501S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PRSRSH87S19H501S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PRSRSH87S19H501S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PRSRSH87S19H501S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L22" s="6">
-        <f>IF(75=0,0,MIN((J22*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="D22" s="5">
+        <f>'Aprile 2026'!AH23+'Maggio 2026'!AI23+'Giugno 2026'!AH23+'Luglio 2026'!AI23+'Agosto 2026'!AI23+'Settembre 2026'!AH23</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>'Aprile 2026'!AJ23+'Maggio 2026'!AK23+'Giugno 2026'!AJ23+'Luglio 2026'!AK23+'Agosto 2026'!AK23+'Settembre 2026'!AJ23</f>
+        <v/>
+      </c>
+      <c r="F22" s="6">
+        <f>IF(75=0,0,MIN((D22*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>La Cyber Security; Cloud e Fog Computing</t>
         </is>
       </c>
-      <c r="N22" s="4" t="n">
+      <c r="H22" s="4" t="n">
         <v>12.41267106976744</v>
       </c>
-      <c r="O22" s="4" t="n">
+      <c r="I22" s="4" t="n">
         <v>6.186176741112714</v>
       </c>
-      <c r="P22" s="7">
-        <f>(N22+O22)*J22*24</f>
+      <c r="J22" s="7">
+        <f>(H22+I22)*D22*24</f>
         <v/>
       </c>
     </row>
@@ -3705,31 +3705,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J23" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("PDDRND75R08H501S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("PDDRND75R08H501S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("PDDRND75R08H501S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("PDDRND75R08H501S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("PDDRND75R08H501S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("PDDRND75R08H501S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K23" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("PDDRND75R08H501S",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("PDDRND75R08H501S",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("PDDRND75R08H501S",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("PDDRND75R08H501S",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("PDDRND75R08H501S",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("PDDRND75R08H501S",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L23" s="6">
-        <f>IF(75=0,0,MIN((J23*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="D23" s="5">
+        <f>'Aprile 2026'!AH24+'Maggio 2026'!AI24+'Giugno 2026'!AH24+'Luglio 2026'!AI24+'Agosto 2026'!AI24+'Settembre 2026'!AH24</f>
+        <v/>
+      </c>
+      <c r="E23" s="5">
+        <f>'Aprile 2026'!AJ24+'Maggio 2026'!AK24+'Giugno 2026'!AJ24+'Luglio 2026'!AK24+'Agosto 2026'!AK24+'Settembre 2026'!AJ24</f>
+        <v/>
+      </c>
+      <c r="F23" s="6">
+        <f>IF(75=0,0,MIN((D23*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Big data e analisi predittiva; Deep Learning e reti neurali</t>
         </is>
       </c>
-      <c r="N23" s="4" t="n">
+      <c r="H23" s="4" t="n">
         <v>11.02898009302326</v>
       </c>
-      <c r="O23" s="4" t="n">
+      <c r="I23" s="4" t="n">
         <v>5.496582132484965</v>
       </c>
-      <c r="P23" s="7">
-        <f>(N23+O23)*J23*24</f>
+      <c r="J23" s="7">
+        <f>(H23+I23)*D23*24</f>
         <v/>
       </c>
     </row>
@@ -3749,31 +3749,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J24" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("RNRFNC99L28H501B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("RNRFNC99L28H501B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("RNRFNC99L28H501B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("RNRFNC99L28H501B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("RNRFNC99L28H501B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("RNRFNC99L28H501B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K24" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("RNRFNC99L28H501B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("RNRFNC99L28H501B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("RNRFNC99L28H501B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("RNRFNC99L28H501B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("RNRFNC99L28H501B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("RNRFNC99L28H501B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L24" s="6">
-        <f>IF(75=0,0,MIN((J24*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="D24" s="5">
+        <f>'Aprile 2026'!AH25+'Maggio 2026'!AI25+'Giugno 2026'!AH25+'Luglio 2026'!AI25+'Agosto 2026'!AI25+'Settembre 2026'!AH25</f>
+        <v/>
+      </c>
+      <c r="E24" s="5">
+        <f>'Aprile 2026'!AJ25+'Maggio 2026'!AK25+'Giugno 2026'!AJ25+'Luglio 2026'!AK25+'Agosto 2026'!AK25+'Settembre 2026'!AJ25</f>
+        <v/>
+      </c>
+      <c r="F24" s="6">
+        <f>IF(75=0,0,MIN((D24*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; I sistemi operativi; Linguaggi di programmazione; Front end base: HTML, CSS, Bootstrap; Back end base: Fondamenti di PHP; Applicazioni dinamiche con PHP e MySql</t>
         </is>
       </c>
-      <c r="N24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>9.858164651162792</v>
       </c>
-      <c r="O24" s="4" t="n">
+      <c r="I24" s="4" t="n">
         <v>1.67451140143258</v>
       </c>
-      <c r="P24" s="7">
-        <f>(N24+O24)*J24*24</f>
+      <c r="J24" s="7">
+        <f>(H24+I24)*D24*24</f>
         <v/>
       </c>
     </row>
@@ -3793,31 +3793,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J25" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("DLRJMY02A20H501A",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("DLRJMY02A20H501A",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("DLRJMY02A20H501A",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("DLRJMY02A20H501A",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("DLRJMY02A20H501A",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("DLRJMY02A20H501A",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K25" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("DLRJMY02A20H501A",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("DLRJMY02A20H501A",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("DLRJMY02A20H501A",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("DLRJMY02A20H501A",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("DLRJMY02A20H501A",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("DLRJMY02A20H501A",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L25" s="6">
-        <f>IF(75=0,0,MIN((J25*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="D25" s="5">
+        <f>'Aprile 2026'!AH26+'Maggio 2026'!AI26+'Giugno 2026'!AH26+'Luglio 2026'!AI26+'Agosto 2026'!AI26+'Settembre 2026'!AH26</f>
+        <v/>
+      </c>
+      <c r="E25" s="5">
+        <f>'Aprile 2026'!AJ26+'Maggio 2026'!AK26+'Giugno 2026'!AJ26+'Luglio 2026'!AK26+'Agosto 2026'!AK26+'Settembre 2026'!AJ26</f>
+        <v/>
+      </c>
+      <c r="F25" s="6">
+        <f>IF(75=0,0,MIN((D25*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Nessuno - i corsi iniziati sono al 100%</t>
         </is>
       </c>
-      <c r="N25" s="4" t="n">
+      <c r="H25" s="4" t="n">
         <v>8.746046511627904</v>
       </c>
-      <c r="O25" s="4" t="n">
+      <c r="I25" s="4" t="n">
         <v>2.093632948739695</v>
       </c>
-      <c r="P25" s="7">
-        <f>(N25+O25)*J25*24</f>
+      <c r="J25" s="7">
+        <f>(H25+I25)*D25*24</f>
         <v/>
       </c>
     </row>
@@ -3837,31 +3837,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J26" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SLPGLC81B17G377J",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SLPGLC81B17G377J",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SLPGLC81B17G377J",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SLPGLC81B17G377J",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SLPGLC81B17G377J",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SLPGLC81B17G377J",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K26" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SLPGLC81B17G377J",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SLPGLC81B17G377J",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SLPGLC81B17G377J",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SLPGLC81B17G377J",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SLPGLC81B17G377J",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SLPGLC81B17G377J",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L26" s="6">
-        <f>IF(75=0,0,MIN((J26*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="D26" s="5">
+        <f>'Aprile 2026'!AH27+'Maggio 2026'!AI27+'Giugno 2026'!AH27+'Luglio 2026'!AI27+'Agosto 2026'!AI27+'Settembre 2026'!AH27</f>
+        <v/>
+      </c>
+      <c r="E26" s="5">
+        <f>'Aprile 2026'!AJ27+'Maggio 2026'!AK27+'Giugno 2026'!AJ27+'Luglio 2026'!AK27+'Agosto 2026'!AK27+'Settembre 2026'!AJ27</f>
+        <v/>
+      </c>
+      <c r="F26" s="6">
+        <f>IF(75=0,0,MIN((D26*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Big data e analisi predittiva; I Big data in ambito finanziario; Gestione avanzata di un Database; Sicurezza e Password Management</t>
         </is>
       </c>
-      <c r="N26" s="4" t="n">
+      <c r="H26" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O26" s="4" t="n">
+      <c r="I26" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P26" s="7">
-        <f>(N26+O26)*J26*24</f>
+      <c r="J26" s="7">
+        <f>(H26+I26)*D26*24</f>
         <v/>
       </c>
     </row>
@@ -3881,31 +3881,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J27" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SLVCMN80D14D086Z",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SLVCMN80D14D086Z",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SLVCMN80D14D086Z",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SLVCMN80D14D086Z",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SLVCMN80D14D086Z",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SLVCMN80D14D086Z",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K27" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SLVCMN80D14D086Z",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SLVCMN80D14D086Z",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SLVCMN80D14D086Z",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SLVCMN80D14D086Z",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SLVCMN80D14D086Z",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SLVCMN80D14D086Z",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="6">
-        <f>IF(75=0,0,MIN((J27*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="D27" s="5">
+        <f>'Aprile 2026'!AH28+'Maggio 2026'!AI28+'Giugno 2026'!AH28+'Luglio 2026'!AI28+'Agosto 2026'!AI28+'Settembre 2026'!AH28</f>
+        <v/>
+      </c>
+      <c r="E27" s="5">
+        <f>'Aprile 2026'!AJ28+'Maggio 2026'!AK28+'Giugno 2026'!AJ28+'Luglio 2026'!AK28+'Agosto 2026'!AK28+'Settembre 2026'!AJ28</f>
+        <v/>
+      </c>
+      <c r="F27" s="6">
+        <f>IF(75=0,0,MIN((D27*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Big data e analisi predittiva; I Big data in ambito finanziario; Database relazionali e linguaggio SQL con PHP; Natural Language Processing con Python; Il Machine Learning con Python; Progettare autorizzazioni e autentificazioni; Gestione avanzata di un Database; Sicurezza e Password Management</t>
         </is>
       </c>
-      <c r="N27" s="4" t="n">
+      <c r="H27" s="4" t="n">
         <v>11.66253823255814</v>
       </c>
-      <c r="O27" s="4" t="n">
+      <c r="I27" s="4" t="n">
         <v>5.812305599793496</v>
       </c>
-      <c r="P27" s="7">
-        <f>(N27+O27)*J27*24</f>
+      <c r="J27" s="7">
+        <f>(H27+I27)*D27*24</f>
         <v/>
       </c>
     </row>
@@ -3925,31 +3925,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J28" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SMBLSS74D47H501E",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SMBLSS74D47H501E",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SMBLSS74D47H501E",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SMBLSS74D47H501E",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SMBLSS74D47H501E",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SMBLSS74D47H501E",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K28" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SMBLSS74D47H501E",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SMBLSS74D47H501E",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SMBLSS74D47H501E",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SMBLSS74D47H501E",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SMBLSS74D47H501E",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SMBLSS74D47H501E",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="6">
-        <f>IF(75=0,0,MIN((J28*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="D28" s="5">
+        <f>'Aprile 2026'!AH29+'Maggio 2026'!AI29+'Giugno 2026'!AH29+'Luglio 2026'!AI29+'Agosto 2026'!AI29+'Settembre 2026'!AH29</f>
+        <v/>
+      </c>
+      <c r="E28" s="5">
+        <f>'Aprile 2026'!AJ29+'Maggio 2026'!AK29+'Giugno 2026'!AJ29+'Luglio 2026'!AK29+'Agosto 2026'!AK29+'Settembre 2026'!AJ29</f>
+        <v/>
+      </c>
+      <c r="F28" s="6">
+        <f>IF(75=0,0,MIN((D28*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Introduzione ai Big Data nelle aziende; Big data e analisi predittiva; Progettare autorizzazioni e autentificazioni</t>
         </is>
       </c>
-      <c r="N28" s="4" t="n">
+      <c r="H28" s="4" t="n">
         <v>10.42583274418605</v>
       </c>
-      <c r="O28" s="4" t="n">
+      <c r="I28" s="4" t="n">
         <v>5.131004531257418</v>
       </c>
-      <c r="P28" s="7">
-        <f>(N28+O28)*J28*24</f>
+      <c r="J28" s="7">
+        <f>(H28+I28)*D28*24</f>
         <v/>
       </c>
     </row>
@@ -3969,31 +3969,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J29" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SVNSLV89A46H501I",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SVNSLV89A46H501I",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SVNSLV89A46H501I",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SVNSLV89A46H501I",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SVNSLV89A46H501I",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SVNSLV89A46H501I",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K29" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SVNSLV89A46H501I",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SVNSLV89A46H501I",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SVNSLV89A46H501I",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SVNSLV89A46H501I",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SVNSLV89A46H501I",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SVNSLV89A46H501I",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="6">
-        <f>IF(75=0,0,MIN((J29*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="D29" s="5">
+        <f>'Aprile 2026'!AH30+'Maggio 2026'!AI30+'Giugno 2026'!AH30+'Luglio 2026'!AI30+'Agosto 2026'!AI30+'Settembre 2026'!AH30</f>
+        <v/>
+      </c>
+      <c r="E29" s="5">
+        <f>'Aprile 2026'!AJ30+'Maggio 2026'!AK30+'Giugno 2026'!AJ30+'Luglio 2026'!AK30+'Agosto 2026'!AK30+'Settembre 2026'!AJ30</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>IF(75=0,0,MIN((D29*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; I sistemi operativi; Linguaggi di programmazione; Back end base: Fondamenti di PHP</t>
         </is>
       </c>
-      <c r="N29" s="4" t="n">
+      <c r="H29" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O29" s="4" t="n">
+      <c r="I29" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P29" s="7">
-        <f>(N29+O29)*J29*24</f>
+      <c r="J29" s="7">
+        <f>(H29+I29)*D29*24</f>
         <v/>
       </c>
     </row>
@@ -4013,31 +4013,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J30" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SCLFPP97S05H501K",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SCLFPP97S05H501K",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SCLFPP97S05H501K",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SCLFPP97S05H501K",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SCLFPP97S05H501K",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SCLFPP97S05H501K",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K30" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SCLFPP97S05H501K",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SCLFPP97S05H501K",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SCLFPP97S05H501K",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SCLFPP97S05H501K",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SCLFPP97S05H501K",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SCLFPP97S05H501K",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="6">
-        <f>IF(75=0,0,MIN((J30*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="D30" s="5">
+        <f>'Aprile 2026'!AH31+'Maggio 2026'!AI31+'Giugno 2026'!AH31+'Luglio 2026'!AI31+'Agosto 2026'!AI31+'Settembre 2026'!AH31</f>
+        <v/>
+      </c>
+      <c r="E30" s="5">
+        <f>'Aprile 2026'!AJ31+'Maggio 2026'!AK31+'Giugno 2026'!AJ31+'Luglio 2026'!AK31+'Agosto 2026'!AK31+'Settembre 2026'!AJ31</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>IF(75=0,0,MIN((D30*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Big Data Analytics con Python e Spark</t>
         </is>
       </c>
-      <c r="N30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>9.858164651162792</v>
       </c>
-      <c r="O30" s="4" t="n">
+      <c r="I30" s="4" t="n">
         <v>1.683757475327303</v>
       </c>
-      <c r="P30" s="7">
-        <f>(N30+O30)*J30*24</f>
+      <c r="J30" s="7">
+        <f>(H30+I30)*D30*24</f>
         <v/>
       </c>
     </row>
@@ -4057,31 +4057,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J31" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("SCRTZN80A09H501I",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("SCRTZN80A09H501I",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("SCRTZN80A09H501I",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("SCRTZN80A09H501I",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("SCRTZN80A09H501I",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("SCRTZN80A09H501I",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K31" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("SCRTZN80A09H501I",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("SCRTZN80A09H501I",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("SCRTZN80A09H501I",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("SCRTZN80A09H501I",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("SCRTZN80A09H501I",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("SCRTZN80A09H501I",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="6">
-        <f>IF(75=0,0,MIN((J31*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="D31" s="5">
+        <f>'Aprile 2026'!AH32+'Maggio 2026'!AI32+'Giugno 2026'!AH32+'Luglio 2026'!AI32+'Agosto 2026'!AI32+'Settembre 2026'!AH32</f>
+        <v/>
+      </c>
+      <c r="E31" s="5">
+        <f>'Aprile 2026'!AJ32+'Maggio 2026'!AK32+'Giugno 2026'!AJ32+'Luglio 2026'!AK32+'Agosto 2026'!AK32+'Settembre 2026'!AJ32</f>
+        <v/>
+      </c>
+      <c r="F31" s="6">
+        <f>IF(75=0,0,MIN((D31*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>GDPR e nuove normative Europee; Big data e analisi predittiva; Database relazionali e linguaggio SQL con PHP; Deep Learning e reti neurali</t>
         </is>
       </c>
-      <c r="N31" s="4" t="n">
+      <c r="H31" s="4" t="n">
         <v>12.24034325581395</v>
       </c>
-      <c r="O31" s="4" t="n">
+      <c r="I31" s="4" t="n">
         <v>6.0163062496053</v>
       </c>
-      <c r="P31" s="7">
-        <f>(N31+O31)*J31*24</f>
+      <c r="J31" s="7">
+        <f>(H31+I31)*D31*24</f>
         <v/>
       </c>
     </row>
@@ -4101,31 +4101,31 @@
           <t>Big Data - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J32" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("STSDNS91B05Z140T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("STSDNS91B05Z140T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("STSDNS91B05Z140T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("STSDNS91B05Z140T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("STSDNS91B05Z140T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("STSDNS91B05Z140T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K32" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("STSDNS91B05Z140T",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("STSDNS91B05Z140T",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("STSDNS91B05Z140T",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("STSDNS91B05Z140T",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("STSDNS91B05Z140T",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("STSDNS91B05Z140T",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L32" s="6">
-        <f>IF(75=0,0,MIN((J32*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="D32" s="5">
+        <f>'Aprile 2026'!AH33+'Maggio 2026'!AI33+'Giugno 2026'!AH33+'Luglio 2026'!AI33+'Agosto 2026'!AI33+'Settembre 2026'!AH33</f>
+        <v/>
+      </c>
+      <c r="E32" s="5">
+        <f>'Aprile 2026'!AJ33+'Maggio 2026'!AK33+'Giugno 2026'!AJ33+'Luglio 2026'!AK33+'Agosto 2026'!AK33+'Settembre 2026'!AJ33</f>
+        <v/>
+      </c>
+      <c r="F32" s="6">
+        <f>IF(75=0,0,MIN((D32*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>I Big data in ambito finanziario; Natural Language Processing con Python</t>
         </is>
       </c>
-      <c r="N32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>10.28898418604651</v>
       </c>
-      <c r="O32" s="4" t="n">
+      <c r="I32" s="4" t="n">
         <v>5.127761382625514</v>
       </c>
-      <c r="P32" s="7">
-        <f>(N32+O32)*J32*24</f>
+      <c r="J32" s="7">
+        <f>(H32+I32)*D32*24</f>
         <v/>
       </c>
     </row>
@@ -4145,31 +4145,31 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J33" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("TRSNDR97M24H501B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("TRSNDR97M24H501B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("TRSNDR97M24H501B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("TRSNDR97M24H501B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("TRSNDR97M24H501B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("TRSNDR97M24H501B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K33" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("TRSNDR97M24H501B",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("TRSNDR97M24H501B",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("TRSNDR97M24H501B",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("TRSNDR97M24H501B",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("TRSNDR97M24H501B",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("TRSNDR97M24H501B",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L33" s="6">
-        <f>IF(75=0,0,MIN((J33*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="D33" s="5">
+        <f>'Aprile 2026'!AH34+'Maggio 2026'!AI34+'Giugno 2026'!AH34+'Luglio 2026'!AI34+'Agosto 2026'!AI34+'Settembre 2026'!AH34</f>
+        <v/>
+      </c>
+      <c r="E33" s="5">
+        <f>'Aprile 2026'!AJ34+'Maggio 2026'!AK34+'Giugno 2026'!AJ34+'Luglio 2026'!AK34+'Agosto 2026'!AK34+'Settembre 2026'!AJ34</f>
+        <v/>
+      </c>
+      <c r="F33" s="6">
+        <f>IF(75=0,0,MIN((D33*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Front end avanzato: JavaScript e jQuery; Applicazioni dinamiche con PHP e MySql</t>
         </is>
       </c>
-      <c r="N33" s="4" t="n">
+      <c r="H33" s="4" t="n">
         <v>10.52720204651162</v>
       </c>
-      <c r="O33" s="4" t="n">
+      <c r="I33" s="4" t="n">
         <v>5.777385318779284</v>
       </c>
-      <c r="P33" s="7">
-        <f>(N33+O33)*J33*24</f>
+      <c r="J33" s="7">
+        <f>(H33+I33)*D33*24</f>
         <v/>
       </c>
     </row>
@@ -4189,32 +4189,35 @@
           <t>La programmazione - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J34" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("TCONNT91H59Z100O",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("TCONNT91H59Z100O",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("TCONNT91H59Z100O",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("TCONNT91H59Z100O",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("TCONNT91H59Z100O",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("TCONNT91H59Z100O",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K34" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("TCONNT91H59Z100O",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("TCONNT91H59Z100O",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("TCONNT91H59Z100O",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("TCONNT91H59Z100O",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("TCONNT91H59Z100O",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("TCONNT91H59Z100O",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L34" s="6">
-        <f>IF(75=0,0,MIN((J34*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="D34" s="5">
+        <f>'Aprile 2026'!AH35+'Maggio 2026'!AI35+'Giugno 2026'!AH35+'Luglio 2026'!AI35+'Agosto 2026'!AI35+'Settembre 2026'!AH35</f>
+        <v/>
+      </c>
+      <c r="E34" s="5">
+        <f>'Aprile 2026'!AJ35+'Maggio 2026'!AK35+'Giugno 2026'!AJ35+'Luglio 2026'!AK35+'Agosto 2026'!AK35+'Settembre 2026'!AJ35</f>
+        <v/>
+      </c>
+      <c r="F34" s="6">
+        <f>IF(75=0,0,MIN((D34*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Nessuno - i corsi iniziati sono al 100%</t>
         </is>
       </c>
-      <c r="N34" s="4" t="n">
+      <c r="H34" s="4" t="n">
         <v>9.731453023255815</v>
       </c>
-      <c r="O34" s="4" t="n">
+      <c r="I34" s="4" t="n">
         <v>4.849926321476056</v>
       </c>
-      <c r="P34" s="7">
-        <f>(N34+O34)*J34*24</f>
-        <v/>
+      <c r="J34" s="7">
+        <f>(H34+I34)*D34*24</f>
+        <v/>
+      </c>
+      <c r="K34" t="n">
+        <v>70242.3</v>
       </c>
     </row>
     <row r="35" ht="20.1" customHeight="1">
@@ -4233,31 +4236,31 @@
           <t>Project Management per il digitale - Tecninf - Fondoconoscenza</t>
         </is>
       </c>
-      <c r="J35" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AH4:AH37,MATCH("VSWSDH86S22Z222H",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AI4:AI37,MATCH("VSWSDH86S22Z222H",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AH4:AH37,MATCH("VSWSDH86S22Z222H",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AI4:AI37,MATCH("VSWSDH86S22Z222H",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AI4:AI37,MATCH("VSWSDH86S22Z222H",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AH4:AH37,MATCH("VSWSDH86S22Z222H",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="K35" s="5">
-        <f>IFERROR(INDEX('Aprile 2026'!AJ4:AJ37,MATCH("VSWSDH86S22Z222H",'Aprile 2026'!B4:B37,0)),0)+IFERROR(INDEX('Maggio 2026'!AK4:AK37,MATCH("VSWSDH86S22Z222H",'Maggio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Giugno 2026'!AJ4:AJ37,MATCH("VSWSDH86S22Z222H",'Giugno 2026'!B4:B37,0)),0)+IFERROR(INDEX('Luglio 2026'!AK4:AK37,MATCH("VSWSDH86S22Z222H",'Luglio 2026'!B4:B37,0)),0)+IFERROR(INDEX('Agosto 2026'!AK4:AK37,MATCH("VSWSDH86S22Z222H",'Agosto 2026'!B4:B37,0)),0)+IFERROR(INDEX('Settembre 2026'!AJ4:AJ37,MATCH("VSWSDH86S22Z222H",'Settembre 2026'!B4:B37,0)),0)</f>
-        <v/>
-      </c>
-      <c r="L35" s="6">
-        <f>IF(75=0,0,MIN((J35*24)/150,1))</f>
-        <v/>
-      </c>
-      <c r="M35" s="3" t="inlineStr">
+      <c r="D35" s="5">
+        <f>'Aprile 2026'!AH36+'Maggio 2026'!AI36+'Giugno 2026'!AH36+'Luglio 2026'!AI36+'Agosto 2026'!AI36+'Settembre 2026'!AH36</f>
+        <v/>
+      </c>
+      <c r="E35" s="5">
+        <f>'Aprile 2026'!AJ36+'Maggio 2026'!AK36+'Giugno 2026'!AJ36+'Luglio 2026'!AK36+'Agosto 2026'!AK36+'Settembre 2026'!AJ36</f>
+        <v/>
+      </c>
+      <c r="F35" s="6">
+        <f>IF(75=0,0,MIN((D35*24)/150,1))</f>
+        <v/>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Influenzare positivamente il clima aziendale</t>
         </is>
       </c>
-      <c r="N35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>11.99198846511628</v>
       </c>
-      <c r="O35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>5.976475500904301</v>
       </c>
-      <c r="P35" s="7">
-        <f>(N35+O35)*J35*24</f>
+      <c r="J35" s="7">
+        <f>(H35+I35)*D35*24</f>
         <v/>
       </c>
     </row>
@@ -4267,16 +4270,16 @@
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="J36" s="9">
+      <c r="D36" s="9">
+        <f>SUM(D3:D35)</f>
+        <v/>
+      </c>
+      <c r="E36" s="9">
+        <f>SUM(E3:E35)</f>
+        <v/>
+      </c>
+      <c r="J36" s="10">
         <f>SUM(J3:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="9">
-        <f>SUM(K3:K35)</f>
-        <v/>
-      </c>
-      <c r="P36" s="10">
-        <f>SUM(P3:P35)</f>
         <v/>
       </c>
     </row>
@@ -4286,10 +4289,14 @@
           <t>TOTALE NON FINANZIATO</t>
         </is>
       </c>
+      <c r="J37" s="10">
+        <f>K34-J36</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>